<commit_message>
Add work remaining guide and branch discoveries
</commit_message>
<xml_diff>
--- a/outputs/branch-registry/Welsh-LDS-Branch-Registry.xlsx
+++ b/outputs/branch-registry/Welsh-LDS-Branch-Registry.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Registry" sheetId="1" r:id="R7455c56524b54a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Rc3f57aa22c6c4e98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R5950bb211a75453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Registry" sheetId="1" r:id="R561ef5d3dcc1478c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="R36afd86074224c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R679939dc41ed49ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -151,19 +151,19 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{A6E1244E-3FDE-4FF8-847A-AF2AC7776DA7}"/>
+  <xltc:person displayName="User" id="{8D653FC7-4EF1-4F17-A7E2-B61C5BA565DD}"/>
 </xltc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BranchRegistryTable" displayName="BranchRegistryTable" ref="A1:N56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BranchRegistryTable" displayName="BranchRegistryTable" ref="A1:N59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Canonical name"/>
     <x:tableColumn id="2" name="Entity type"/>
     <x:tableColumn id="3" name="Known variants"/>
     <x:tableColumn id="4" name="Earliest year"/>
     <x:tableColumn id="5" name="Latest year"/>
-    <x:tableColumn id="6" name="Local CD index"/>
+    <x:tableColumn id="6" name="Local record evidence"/>
     <x:tableColumn id="7" name="Recovered note"/>
     <x:tableColumn id="8" name="FamilySearch catalog"/>
     <x:tableColumn id="9" name="Comparison status"/>
@@ -178,7 +178,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BranchEvidenceTable" displayName="BranchEvidenceTable" ref="A1:I106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BranchEvidenceTable" displayName="BranchEvidenceTable" ref="A1:I112" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Raw name as found"/>
     <x:tableColumn id="2" name="Proposed canonical name"/>
@@ -422,7 +422,7 @@
         <x:v>Latest year</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Local CD index</x:v>
+        <x:v>Local record evidence</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
         <x:v>Recovered note</x:v>
@@ -478,7 +478,7 @@
         <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J2" s="5" t="str">
-        <x:v>CD 25; LR 10468 7; Wales2Utah research note</x:v>
+        <x:v>CD 25; LR 10468 7; CD 62; general minutes; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K2" s="5" t="str"/>
       <x:c r="L2" s="5" t="str"/>
@@ -1130,7 +1130,9 @@
       <x:c r="B20" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="str"/>
+      <x:c r="C20" s="5" t="str">
+        <x:v>Gymmer</x:v>
+      </x:c>
       <x:c r="D20" s="6" t="n">
         <x:v>1850</x:v>
       </x:c>
@@ -1150,7 +1152,7 @@
         <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J20" s="5" t="str">
-        <x:v>CD 9; LR 11152 23</x:v>
+        <x:v>CD 9; LR 11152 23; CD 59; meeting transcription checklist</x:v>
       </x:c>
       <x:c r="K20" s="5" t="str"/>
       <x:c r="L20" s="5" t="str"/>
@@ -1921,32 +1923,28 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="4" t="str">
-        <x:v>Pontlanfraith</x:v>
+        <x:v>Pen-y-Darran</x:v>
       </x:c>
       <x:c r="B42" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C42" s="5" t="str"/>
-      <x:c r="D42" s="6" t="n">
-        <x:v>1947</x:v>
-      </x:c>
-      <x:c r="E42" s="6" t="n">
-        <x:v>1947</x:v>
-      </x:c>
+      <x:c r="D42" s="6"/>
+      <x:c r="E42" s="6"/>
       <x:c r="F42" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G42" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H42" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I42" s="5" t="str">
-        <x:v>Research note only</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J42" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 36; two-page baptism list</x:v>
       </x:c>
       <x:c r="K42" s="5" t="str"/>
       <x:c r="L42" s="5" t="str"/>
@@ -1957,17 +1955,17 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="4" t="str">
-        <x:v>Pontypridd</x:v>
+        <x:v>Pontlanfraith</x:v>
       </x:c>
       <x:c r="B43" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C43" s="5" t="str"/>
       <x:c r="D43" s="6" t="n">
-        <x:v>1877</x:v>
+        <x:v>1947</x:v>
       </x:c>
       <x:c r="E43" s="6" t="n">
-        <x:v>1895</x:v>
+        <x:v>1947</x:v>
       </x:c>
       <x:c r="F43" s="4" t="str">
         <x:v>No</x:v>
@@ -1993,17 +1991,17 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="4" t="str">
-        <x:v>Rhymney</x:v>
+        <x:v>Pontypool</x:v>
       </x:c>
       <x:c r="B44" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C44" s="5" t="str"/>
       <x:c r="D44" s="6" t="n">
-        <x:v>1850</x:v>
+        <x:v>1857</x:v>
       </x:c>
       <x:c r="E44" s="6" t="n">
-        <x:v>1887</x:v>
+        <x:v>1884</x:v>
       </x:c>
       <x:c r="F44" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2018,7 +2016,7 @@
         <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J44" s="5" t="str">
-        <x:v>CD 20; LR 12451 7</x:v>
+        <x:v>CD 62; general minutes</x:v>
       </x:c>
       <x:c r="K44" s="5" t="str"/>
       <x:c r="L44" s="5" t="str"/>
@@ -2029,129 +2027,127 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="4" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Pontypridd</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C45" s="5" t="str"/>
       <x:c r="D45" s="6" t="n">
-        <x:v>1851</x:v>
+        <x:v>1877</x:v>
       </x:c>
       <x:c r="E45" s="6" t="n">
-        <x:v>1883</x:v>
+        <x:v>1895</x:v>
       </x:c>
       <x:c r="F45" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G45" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H45" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I45" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J45" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
+        <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K45" s="5" t="str"/>
       <x:c r="L45" s="5" t="str"/>
       <x:c r="M45" s="5" t="str">
         <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
       </x:c>
-      <x:c r="N45" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
+      <x:c r="N45" s="5" t="str"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="4" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Rhymney</x:v>
       </x:c>
       <x:c r="B46" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C46" s="5" t="str"/>
       <x:c r="D46" s="6" t="n">
-        <x:v>1853</x:v>
+        <x:v>1850</x:v>
       </x:c>
       <x:c r="E46" s="6" t="n">
-        <x:v>1859</x:v>
+        <x:v>1887</x:v>
       </x:c>
       <x:c r="F46" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G46" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="H46" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I46" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J46" s="5" t="str">
-        <x:v>Film 104171 item 6</x:v>
+        <x:v>CD 20; LR 12451 7</x:v>
       </x:c>
       <x:c r="K46" s="5" t="str"/>
       <x:c r="L46" s="5" t="str"/>
       <x:c r="M46" s="5" t="str">
         <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
       </x:c>
-      <x:c r="N46" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104171</x:v>
-      </x:c>
+      <x:c r="N46" s="5" t="str"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="4" t="str">
-        <x:v>Swansea</x:v>
+        <x:v>Rhymney English</x:v>
       </x:c>
       <x:c r="B47" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C47" s="5" t="str"/>
       <x:c r="D47" s="6" t="n">
-        <x:v>1872</x:v>
+        <x:v>1851</x:v>
       </x:c>
       <x:c r="E47" s="6" t="n">
-        <x:v>1879</x:v>
+        <x:v>1883</x:v>
       </x:c>
       <x:c r="F47" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G47" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="H47" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="I47" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J47" s="5" t="str">
-        <x:v>CD 32; LR 8863 7</x:v>
+        <x:v>Film 104172 Items 7-8</x:v>
       </x:c>
       <x:c r="K47" s="5" t="str"/>
       <x:c r="L47" s="5" t="str"/>
       <x:c r="M47" s="5" t="str">
         <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
       </x:c>
-      <x:c r="N47" s="5" t="str"/>
+      <x:c r="N47" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="4" t="str">
-        <x:v>Treboeth</x:v>
+        <x:v>Stepaside</x:v>
       </x:c>
       <x:c r="B48" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str"/>
       <x:c r="D48" s="6" t="n">
-        <x:v>1844</x:v>
+        <x:v>1858</x:v>
       </x:c>
       <x:c r="E48" s="6" t="n">
-        <x:v>1880</x:v>
+        <x:v>1860</x:v>
       </x:c>
       <x:c r="F48" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2160,37 +2156,37 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="H48" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I48" s="5" t="str">
-        <x:v>Matched: FamilySearch and local CD</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J48" s="5" t="str">
-        <x:v>CD 16; LR 228 7; Film 104172 Item 1</x:v>
+        <x:v>CD 44; LR 12727 11; general minutes</x:v>
       </x:c>
       <x:c r="K48" s="5" t="str"/>
       <x:c r="L48" s="5" t="str"/>
-      <x:c r="M48" s="5" t="str"/>
-      <x:c r="N48" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
+      <x:c r="M48" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N48" s="5" t="str"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="4" t="str">
-        <x:v>Tredegar</x:v>
+        <x:v>Sutton Mountain</x:v>
       </x:c>
       <x:c r="B49" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str"/>
       <x:c r="D49" s="6" t="n">
-        <x:v>1844</x:v>
+        <x:v>1853</x:v>
       </x:c>
       <x:c r="E49" s="6" t="n">
-        <x:v>1883</x:v>
+        <x:v>1859</x:v>
       </x:c>
       <x:c r="F49" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G49" s="4" t="str">
         <x:v>No</x:v>
@@ -2199,31 +2195,33 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I49" s="5" t="str">
-        <x:v>Matched: FamilySearch and local CD</x:v>
+        <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J49" s="5" t="str">
-        <x:v>CD 5; LR 164 7; Film 104172 Items 2-3</x:v>
+        <x:v>Film 104171 item 6</x:v>
       </x:c>
       <x:c r="K49" s="5" t="str"/>
       <x:c r="L49" s="5" t="str"/>
-      <x:c r="M49" s="5" t="str"/>
+      <x:c r="M49" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
       <x:c r="N49" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104171</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="4" t="str">
-        <x:v>Treforest</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="B50" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str"/>
       <x:c r="D50" s="6" t="n">
-        <x:v>1851</x:v>
+        <x:v>1852</x:v>
       </x:c>
       <x:c r="E50" s="6" t="n">
-        <x:v>1873</x:v>
+        <x:v>1879</x:v>
       </x:c>
       <x:c r="F50" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2232,37 +2230,37 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="H50" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I50" s="5" t="str">
-        <x:v>Matched: FamilySearch and local CD</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J50" s="5" t="str">
-        <x:v>CD 30; LR 12886 7; Film 104172 Item 4</x:v>
+        <x:v>CD 32; LR 8863 7; CD 61; general minutes</x:v>
       </x:c>
       <x:c r="K50" s="5" t="str"/>
       <x:c r="L50" s="5" t="str"/>
-      <x:c r="M50" s="5" t="str"/>
-      <x:c r="N50" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
+      <x:c r="M50" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N50" s="5" t="str"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="4" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Treboeth</x:v>
       </x:c>
       <x:c r="B51" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str"/>
       <x:c r="D51" s="6" t="n">
-        <x:v>1875</x:v>
+        <x:v>1844</x:v>
       </x:c>
       <x:c r="E51" s="6" t="n">
-        <x:v>1882</x:v>
+        <x:v>1880</x:v>
       </x:c>
       <x:c r="F51" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G51" s="4" t="str">
         <x:v>No</x:v>
@@ -2271,36 +2269,34 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I51" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J51" s="5" t="str">
-        <x:v>Film 104168 Item 13; Film 104172 Item 6</x:v>
+        <x:v>CD 16; LR 228 7; Film 104172 Item 1</x:v>
       </x:c>
       <x:c r="K51" s="5" t="str"/>
       <x:c r="L51" s="5" t="str"/>
-      <x:c r="M51" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M51" s="5" t="str"/>
       <x:c r="N51" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168; https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="4" t="str">
-        <x:v>Trinant</x:v>
+        <x:v>Tredegar</x:v>
       </x:c>
       <x:c r="B52" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str"/>
       <x:c r="D52" s="6" t="n">
-        <x:v>1849</x:v>
+        <x:v>1844</x:v>
       </x:c>
       <x:c r="E52" s="6" t="n">
-        <x:v>1853</x:v>
+        <x:v>1883</x:v>
       </x:c>
       <x:c r="F52" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G52" s="4" t="str">
         <x:v>No</x:v>
@@ -2309,33 +2305,31 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I52" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J52" s="5" t="str">
-        <x:v>Film 104172 Item 6</x:v>
+        <x:v>CD 5; LR 164 7; Film 104172 Items 2-3</x:v>
       </x:c>
       <x:c r="K52" s="5" t="str"/>
       <x:c r="L52" s="5" t="str"/>
-      <x:c r="M52" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M52" s="5" t="str"/>
       <x:c r="N52" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="4" t="str">
-        <x:v>Twyn-yr-Odyn</x:v>
+        <x:v>Treforest</x:v>
       </x:c>
       <x:c r="B53" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str"/>
       <x:c r="D53" s="6" t="n">
-        <x:v>1847</x:v>
+        <x:v>1851</x:v>
       </x:c>
       <x:c r="E53" s="6" t="n">
-        <x:v>1901</x:v>
+        <x:v>1873</x:v>
       </x:c>
       <x:c r="F53" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2350,7 +2344,7 @@
         <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J53" s="5" t="str">
-        <x:v>CD 33; LR 165 7; Film 104172 Items 9-10</x:v>
+        <x:v>CD 30; LR 12886 7; Film 104172 Item 4</x:v>
       </x:c>
       <x:c r="K53" s="5" t="str"/>
       <x:c r="L53" s="5" t="str"/>
@@ -2361,17 +2355,17 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="4" t="str">
-        <x:v>Twyncarno</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="B54" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str"/>
       <x:c r="D54" s="6" t="n">
-        <x:v>1851</x:v>
+        <x:v>1875</x:v>
       </x:c>
       <x:c r="E54" s="6" t="n">
-        <x:v>1883</x:v>
+        <x:v>1882</x:v>
       </x:c>
       <x:c r="F54" s="4" t="str">
         <x:v>No</x:v>
@@ -2386,7 +2380,7 @@
         <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J54" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
+        <x:v>Film 104168 Item 13; Film 104172 Item 6</x:v>
       </x:c>
       <x:c r="K54" s="5" t="str"/>
       <x:c r="L54" s="5" t="str"/>
@@ -2394,28 +2388,28 @@
         <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
       </x:c>
       <x:c r="N54" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168; https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="4" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Trinant</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
-        <x:v>Conference</x:v>
+        <x:v>Branch</x:v>
       </x:c>
       <x:c r="C55" s="5" t="str"/>
       <x:c r="D55" s="6" t="n">
-        <x:v>1850</x:v>
+        <x:v>1849</x:v>
       </x:c>
       <x:c r="E55" s="6" t="n">
-        <x:v>1922</x:v>
+        <x:v>1853</x:v>
       </x:c>
       <x:c r="F55" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G55" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H55" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2424,7 +2418,7 @@
         <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J55" s="5" t="str">
-        <x:v>Wales2Utah research note; Film 104172 Item 11</x:v>
+        <x:v>Film 104172 Item 6</x:v>
       </x:c>
       <x:c r="K55" s="5" t="str"/>
       <x:c r="L55" s="5" t="str"/>
@@ -2437,20 +2431,20 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="4" t="str">
-        <x:v>Ystrad</x:v>
+        <x:v>Twyn-yr-Odyn</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str"/>
       <x:c r="D56" s="6" t="n">
-        <x:v>1885</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="E56" s="6" t="n">
-        <x:v>1911</x:v>
+        <x:v>1901</x:v>
       </x:c>
       <x:c r="F56" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G56" s="4" t="str">
         <x:v>No</x:v>
@@ -2459,29 +2453,141 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I56" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J56" s="5" t="str">
-        <x:v>Film 104172 Item 12</x:v>
+        <x:v>CD 33; LR 165 7; Film 104172 Items 9-10</x:v>
       </x:c>
       <x:c r="K56" s="5" t="str"/>
       <x:c r="L56" s="5" t="str"/>
-      <x:c r="M56" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M56" s="5" t="str"/>
       <x:c r="N56" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="4" t="str">
+        <x:v>Twyncarno</x:v>
+      </x:c>
+      <x:c r="B57" s="4" t="str">
+        <x:v>Branch</x:v>
+      </x:c>
+      <x:c r="C57" s="5" t="str"/>
+      <x:c r="D57" s="6" t="n">
+        <x:v>1851</x:v>
+      </x:c>
+      <x:c r="E57" s="6" t="n">
+        <x:v>1883</x:v>
+      </x:c>
+      <x:c r="F57" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G57" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H57" s="4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I57" s="5" t="str">
+        <x:v>FamilySearch only / locate local record</x:v>
+      </x:c>
+      <x:c r="J57" s="5" t="str">
+        <x:v>Film 104172 Items 7-8</x:v>
+      </x:c>
+      <x:c r="K57" s="5" t="str"/>
+      <x:c r="L57" s="5" t="str"/>
+      <x:c r="M57" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N57" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="4" t="str">
+        <x:v>Welsh Conference</x:v>
+      </x:c>
+      <x:c r="B58" s="4" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="C58" s="5" t="str"/>
+      <x:c r="D58" s="6" t="n">
+        <x:v>1850</x:v>
+      </x:c>
+      <x:c r="E58" s="6" t="n">
+        <x:v>1922</x:v>
+      </x:c>
+      <x:c r="F58" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G58" s="4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H58" s="4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I58" s="5" t="str">
+        <x:v>FamilySearch only / locate local record</x:v>
+      </x:c>
+      <x:c r="J58" s="5" t="str">
+        <x:v>Wales2Utah research note; Film 104172 Item 11</x:v>
+      </x:c>
+      <x:c r="K58" s="5" t="str"/>
+      <x:c r="L58" s="5" t="str"/>
+      <x:c r="M58" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N58" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="4" t="str">
+        <x:v>Ystrad</x:v>
+      </x:c>
+      <x:c r="B59" s="4" t="str">
+        <x:v>Branch</x:v>
+      </x:c>
+      <x:c r="C59" s="5" t="str"/>
+      <x:c r="D59" s="6" t="n">
+        <x:v>1885</x:v>
+      </x:c>
+      <x:c r="E59" s="6" t="n">
+        <x:v>1911</x:v>
+      </x:c>
+      <x:c r="F59" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G59" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H59" s="4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I59" s="5" t="str">
+        <x:v>FamilySearch only / locate local record</x:v>
+      </x:c>
+      <x:c r="J59" s="5" t="str">
+        <x:v>Film 104172 Item 12</x:v>
+      </x:c>
+      <x:c r="K59" s="5" t="str"/>
+      <x:c r="L59" s="5" t="str"/>
+      <x:c r="M59" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N59" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="I2:I56">
+  <x:conditionalFormatting sqref="I2:I59">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FamilySearch only"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Local CD only"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Matched"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58a059b25c9d43e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd152988f60f24a67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3314,150 +3420,146 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="5" t="str">
-        <x:v>Abersycan (1887-1889)</x:v>
+        <x:v>Pen-y-Darran</x:v>
       </x:c>
       <x:c r="B36" s="5" t="str">
-        <x:v>Abersychan</x:v>
+        <x:v>Pen-y-Darran</x:v>
       </x:c>
       <x:c r="C36" s="5" t="str"/>
       <x:c r="D36" s="5" t="str"/>
       <x:c r="E36" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F36" s="5" t="str">
-        <x:v>1887-1889</x:v>
-      </x:c>
+        <x:v>2007 meeting transcription checklist</x:v>
+      </x:c>
+      <x:c r="F36" s="5" t="str"/>
       <x:c r="G36" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 36; two-page baptism list</x:v>
       </x:c>
       <x:c r="H36" s="5" t="str"/>
       <x:c r="I36" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersycan_(1887-1889).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\Wales\Welsh Church Records 1847-1899\ORIGINAL CDs (Orig Welsh 1800s Records)</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="5" t="str">
-        <x:v>Abersychan (1848-1876)</x:v>
+        <x:v>Gymmer</x:v>
       </x:c>
       <x:c r="B37" s="5" t="str">
-        <x:v>Abersychan</x:v>
+        <x:v>Cymmer</x:v>
       </x:c>
       <x:c r="C37" s="5" t="str"/>
       <x:c r="D37" s="5" t="str"/>
       <x:c r="E37" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F37" s="5" t="str">
-        <x:v>1848-1876</x:v>
+        <x:v>1852-1857; 1863</x:v>
       </x:c>
       <x:c r="G37" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 59; meeting transcription checklist</x:v>
       </x:c>
       <x:c r="H37" s="5" t="str"/>
       <x:c r="I37" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersychan_(1848-1876).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\Wales\Welsh Church Records 1847-1899\ORIGINAL CDs (Orig Welsh 1800s Records)</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="5" t="str">
-        <x:v>Abertawe (see Swansea)</x:v>
+        <x:v>Stepaside</x:v>
       </x:c>
       <x:c r="B38" s="5" t="str">
-        <x:v>Abertawe</x:v>
-      </x:c>
-      <x:c r="C38" s="5" t="str">
-        <x:v>Swansea</x:v>
-      </x:c>
-      <x:c r="D38" s="5" t="str">
-        <x:v>See Swansea — possible rename, merger, transfer, or cross-reference; verify before classifying.</x:v>
-      </x:c>
+        <x:v>Stepaside</x:v>
+      </x:c>
+      <x:c r="C38" s="5" t="str"/>
+      <x:c r="D38" s="5" t="str"/>
       <x:c r="E38" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F38" s="5" t="str"/>
+        <x:v>2007 meeting transcription checklist</x:v>
+      </x:c>
+      <x:c r="F38" s="5" t="str">
+        <x:v>1858-1860</x:v>
+      </x:c>
       <x:c r="G38" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 44; LR 12727 11; general minutes</x:v>
       </x:c>
       <x:c r="H38" s="5" t="str"/>
       <x:c r="I38" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertawe_(see_Swansea).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\Wales\Welsh Church Records 1847-1899\ORIGINAL CDs (Orig Welsh 1800s Records)</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="5" t="str">
-        <x:v>Abertillery (1861-1866)</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="B39" s="5" t="str">
-        <x:v>Abertillery</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="C39" s="5" t="str"/>
       <x:c r="D39" s="5" t="str"/>
       <x:c r="E39" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F39" s="5" t="str">
-        <x:v>1861-1866</x:v>
+        <x:v>1852-1854</x:v>
       </x:c>
       <x:c r="G39" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 61; general minutes</x:v>
       </x:c>
       <x:c r="H39" s="5" t="str"/>
       <x:c r="I39" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertillery_(1861-1866).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\Wales\Welsh Church Records 1847-1899\ORIGINAL CDs (Orig Welsh 1800s Records)</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="5" t="str">
-        <x:v>Alltwen (1849-1859)</x:v>
+        <x:v>Pontypool</x:v>
       </x:c>
       <x:c r="B40" s="5" t="str">
-        <x:v>Alltwen</x:v>
+        <x:v>Pontypool</x:v>
       </x:c>
       <x:c r="C40" s="5" t="str"/>
       <x:c r="D40" s="5" t="str"/>
       <x:c r="E40" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F40" s="5" t="str">
-        <x:v>1849-1859</x:v>
+        <x:v>1857-1884</x:v>
       </x:c>
       <x:c r="G40" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 62; general minutes</x:v>
       </x:c>
       <x:c r="H40" s="5" t="str"/>
       <x:c r="I40" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Alltwen_(1849-1859).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\Wales\Welsh Church Records 1847-1899\ORIGINAL CDs (Orig Welsh 1800s Records)</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="5" t="str">
-        <x:v>Brechfa (1846-1868)</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="B41" s="5" t="str">
-        <x:v>Brechfa</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="C41" s="5" t="str"/>
       <x:c r="D41" s="5" t="str"/>
       <x:c r="E41" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F41" s="5" t="str">
-        <x:v>1846-1868</x:v>
+        <x:v>1889</x:v>
       </x:c>
       <x:c r="G41" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 62; general minutes</x:v>
       </x:c>
       <x:c r="H41" s="5" t="str"/>
       <x:c r="I41" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Brechfa_(1846-1868).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\Wales\Welsh Church Records 1847-1899\ORIGINAL CDs (Orig Welsh 1800s Records)</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="5" t="str">
-        <x:v>Cardiff (1849-1855)</x:v>
+        <x:v>Abersycan (1887-1889)</x:v>
       </x:c>
       <x:c r="B42" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="C42" s="5" t="str"/>
       <x:c r="D42" s="5" t="str"/>
@@ -3465,22 +3567,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F42" s="5" t="str">
-        <x:v>1849-1855</x:v>
+        <x:v>1887-1889</x:v>
       </x:c>
       <x:c r="G42" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H42" s="5" t="str"/>
       <x:c r="I42" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1849-1855).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersycan_(1887-1889).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="5" t="str">
-        <x:v>Cardiff (1854-1876)</x:v>
+        <x:v>Abersychan (1848-1876)</x:v>
       </x:c>
       <x:c r="B43" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="C43" s="5" t="str"/>
       <x:c r="D43" s="5" t="str"/>
@@ -3488,45 +3590,47 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F43" s="5" t="str">
-        <x:v>1854-1876</x:v>
+        <x:v>1848-1876</x:v>
       </x:c>
       <x:c r="G43" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H43" s="5" t="str"/>
       <x:c r="I43" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1854-1876).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersychan_(1848-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="5" t="str">
-        <x:v>Cardiff (1931-1947)</x:v>
+        <x:v>Abertawe (see Swansea)</x:v>
       </x:c>
       <x:c r="B44" s="5" t="str">
-        <x:v>Cardiff</x:v>
-      </x:c>
-      <x:c r="C44" s="5" t="str"/>
-      <x:c r="D44" s="5" t="str"/>
+        <x:v>Abertawe</x:v>
+      </x:c>
+      <x:c r="C44" s="5" t="str">
+        <x:v>Swansea</x:v>
+      </x:c>
+      <x:c r="D44" s="5" t="str">
+        <x:v>See Swansea — possible rename, merger, transfer, or cross-reference; verify before classifying.</x:v>
+      </x:c>
       <x:c r="E44" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F44" s="5" t="str">
-        <x:v>1931-1947</x:v>
-      </x:c>
+      <x:c r="F44" s="5" t="str"/>
       <x:c r="G44" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H44" s="5" t="str"/>
       <x:c r="I44" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1931-1947).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertawe_(see_Swansea).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="5" t="str">
-        <x:v>Cardiff (Early to 1917, 1919)</x:v>
+        <x:v>Abertillery (1861-1866)</x:v>
       </x:c>
       <x:c r="B45" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Abertillery</x:v>
       </x:c>
       <x:c r="C45" s="5" t="str"/>
       <x:c r="D45" s="5" t="str"/>
@@ -3534,64 +3638,68 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F45" s="5" t="str">
-        <x:v>1917-1919</x:v>
+        <x:v>1861-1866</x:v>
       </x:c>
       <x:c r="G45" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H45" s="5" t="str"/>
       <x:c r="I45" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(Early_to_1917,_1919).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertillery_(1861-1866).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="5" t="str">
-        <x:v>Cardiff Branch</x:v>
+        <x:v>Alltwen (1849-1859)</x:v>
       </x:c>
       <x:c r="B46" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Alltwen</x:v>
       </x:c>
       <x:c r="C46" s="5" t="str"/>
       <x:c r="D46" s="5" t="str"/>
       <x:c r="E46" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F46" s="5" t="str"/>
+      <x:c r="F46" s="5" t="str">
+        <x:v>1849-1859</x:v>
+      </x:c>
       <x:c r="G46" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H46" s="5" t="str"/>
       <x:c r="I46" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_Branch.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Alltwen_(1849-1859).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Brechfa (1846-1868)</x:v>
       </x:c>
       <x:c r="B47" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Brechfa</x:v>
       </x:c>
       <x:c r="C47" s="5" t="str"/>
       <x:c r="D47" s="5" t="str"/>
       <x:c r="E47" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F47" s="5" t="str"/>
+      <x:c r="F47" s="5" t="str">
+        <x:v>1846-1868</x:v>
+      </x:c>
       <x:c r="G47" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H47" s="5" t="str"/>
       <x:c r="I47" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Castell_Nedd_(Neath).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Brechfa_(1846-1868).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="5" t="str">
-        <x:v>Cefncoed-y-Cymar (1847-1864)</x:v>
+        <x:v>Cardiff (1849-1855)</x:v>
       </x:c>
       <x:c r="B48" s="5" t="str">
-        <x:v>Cefn Coed-y-Cymmer</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str"/>
       <x:c r="D48" s="5" t="str"/>
@@ -3599,22 +3707,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F48" s="5" t="str">
-        <x:v>1847-1864</x:v>
+        <x:v>1849-1855</x:v>
       </x:c>
       <x:c r="G48" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H48" s="5" t="str"/>
       <x:c r="I48" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cefncoed-y-Cymar_(1847-1864).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1849-1855).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="5" t="str">
-        <x:v>Coal Brock Vale (1856-1867)</x:v>
+        <x:v>Cardiff (1854-1876)</x:v>
       </x:c>
       <x:c r="B49" s="5" t="str">
-        <x:v>Coalbrookvale</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str"/>
       <x:c r="D49" s="5" t="str"/>
@@ -3622,22 +3730,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F49" s="5" t="str">
-        <x:v>1856-1867</x:v>
+        <x:v>1854-1876</x:v>
       </x:c>
       <x:c r="G49" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H49" s="5" t="str"/>
       <x:c r="I49" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Coal_Brock_Vale_(1856-1867).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1854-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="5" t="str">
-        <x:v>Cog (1848-1876)</x:v>
+        <x:v>Cardiff (1931-1947)</x:v>
       </x:c>
       <x:c r="B50" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str"/>
       <x:c r="D50" s="5" t="str"/>
@@ -3645,22 +3753,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F50" s="5" t="str">
-        <x:v>1848-1876</x:v>
+        <x:v>1931-1947</x:v>
       </x:c>
       <x:c r="G50" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H50" s="5" t="str"/>
       <x:c r="I50" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cog_(1848-1876).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1931-1947).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="5" t="str">
-        <x:v>Crumlin (1857-1862)</x:v>
+        <x:v>Cardiff (Early to 1917, 1919)</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
-        <x:v>Crumlin</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str"/>
       <x:c r="D51" s="5" t="str"/>
@@ -3668,45 +3776,43 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F51" s="5" t="str">
-        <x:v>1857-1862</x:v>
+        <x:v>1917-1919</x:v>
       </x:c>
       <x:c r="G51" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H51" s="5" t="str"/>
       <x:c r="I51" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Crumlin_(1857-1862).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(Early_to_1917,_1919).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="5" t="str">
-        <x:v>Cuffern Mountain (1849-1876)</x:v>
+        <x:v>Cardiff Branch</x:v>
       </x:c>
       <x:c r="B52" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str"/>
       <x:c r="D52" s="5" t="str"/>
       <x:c r="E52" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F52" s="5" t="str">
-        <x:v>1849-1876</x:v>
-      </x:c>
+      <x:c r="F52" s="5" t="str"/>
       <x:c r="G52" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H52" s="5" t="str"/>
       <x:c r="I52" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cuffern_Mountain_(1849-1876).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_Branch.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="5" t="str">
-        <x:v>Cwm Celin</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="B53" s="5" t="str">
-        <x:v>Cwm Celyn</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str"/>
       <x:c r="D53" s="5" t="str"/>
@@ -3719,78 +3825,84 @@
       </x:c>
       <x:c r="H53" s="5" t="str"/>
       <x:c r="I53" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwm_Celin.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Castell_Nedd_(Neath).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="5" t="str">
-        <x:v>Cwn Tillery</x:v>
+        <x:v>Cefncoed-y-Cymar (1847-1864)</x:v>
       </x:c>
       <x:c r="B54" s="5" t="str">
-        <x:v>Cwmtillery</x:v>
+        <x:v>Cefn Coed-y-Cymmer</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str"/>
       <x:c r="D54" s="5" t="str"/>
       <x:c r="E54" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F54" s="5" t="str"/>
+      <x:c r="F54" s="5" t="str">
+        <x:v>1847-1864</x:v>
+      </x:c>
       <x:c r="G54" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H54" s="5" t="str"/>
       <x:c r="I54" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwn_Tillery.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cefncoed-y-Cymar_(1847-1864).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="5" t="str">
-        <x:v>Dinas</x:v>
+        <x:v>Coal Brock Vale (1856-1867)</x:v>
       </x:c>
       <x:c r="B55" s="5" t="str">
-        <x:v>Dinas</x:v>
+        <x:v>Coalbrookvale</x:v>
       </x:c>
       <x:c r="C55" s="5" t="str"/>
       <x:c r="D55" s="5" t="str"/>
       <x:c r="E55" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F55" s="5" t="str"/>
+      <x:c r="F55" s="5" t="str">
+        <x:v>1856-1867</x:v>
+      </x:c>
       <x:c r="G55" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H55" s="5" t="str"/>
       <x:c r="I55" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dinas.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Coal_Brock_Vale_(1856-1867).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="5" t="str">
-        <x:v>Dowlais</x:v>
+        <x:v>Cog (1848-1876)</x:v>
       </x:c>
       <x:c r="B56" s="5" t="str">
-        <x:v>Dowlais</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str"/>
       <x:c r="D56" s="5" t="str"/>
       <x:c r="E56" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F56" s="5" t="str"/>
+      <x:c r="F56" s="5" t="str">
+        <x:v>1848-1876</x:v>
+      </x:c>
       <x:c r="G56" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H56" s="5" t="str"/>
       <x:c r="I56" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cog_(1848-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="5" t="str">
-        <x:v>Dowlais (1851-1872)</x:v>
+        <x:v>Crumlin (1857-1862)</x:v>
       </x:c>
       <x:c r="B57" s="5" t="str">
-        <x:v>Dowlais</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="C57" s="5" t="str"/>
       <x:c r="D57" s="5" t="str"/>
@@ -3798,43 +3910,45 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F57" s="5" t="str">
-        <x:v>1851-1872</x:v>
+        <x:v>1857-1862</x:v>
       </x:c>
       <x:c r="G57" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H57" s="5" t="str"/>
       <x:c r="I57" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais_(1851-1872).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Crumlin_(1857-1862).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="5" t="str">
-        <x:v>Ebbro Vale</x:v>
+        <x:v>Cuffern Mountain (1849-1876)</x:v>
       </x:c>
       <x:c r="B58" s="5" t="str">
-        <x:v>Ebbw Vale</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str"/>
       <x:c r="D58" s="5" t="str"/>
       <x:c r="E58" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F58" s="5" t="str"/>
+      <x:c r="F58" s="5" t="str">
+        <x:v>1849-1876</x:v>
+      </x:c>
       <x:c r="G58" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H58" s="5" t="str"/>
       <x:c r="I58" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ebbro_Vale.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cuffern_Mountain_(1849-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="5" t="str">
-        <x:v>Ffestiniog</x:v>
+        <x:v>Cwm Celin</x:v>
       </x:c>
       <x:c r="B59" s="5" t="str">
-        <x:v>Ffestiniog</x:v>
+        <x:v>Cwm Celyn</x:v>
       </x:c>
       <x:c r="C59" s="5" t="str"/>
       <x:c r="D59" s="5" t="str"/>
@@ -3847,15 +3961,15 @@
       </x:c>
       <x:c r="H59" s="5" t="str"/>
       <x:c r="I59" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ffestiniog.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwm_Celin.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="5" t="str">
-        <x:v>Georgetown</x:v>
+        <x:v>Cwn Tillery</x:v>
       </x:c>
       <x:c r="B60" s="5" t="str">
-        <x:v>Georgetown</x:v>
+        <x:v>Cwmtillery</x:v>
       </x:c>
       <x:c r="C60" s="5" t="str"/>
       <x:c r="D60" s="5" t="str"/>
@@ -3868,15 +3982,15 @@
       </x:c>
       <x:c r="H60" s="5" t="str"/>
       <x:c r="I60" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Georgetown.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwn_Tillery.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="5" t="str">
-        <x:v>Gilwern</x:v>
+        <x:v>Dinas</x:v>
       </x:c>
       <x:c r="B61" s="5" t="str">
-        <x:v>Gilwern</x:v>
+        <x:v>Dinas</x:v>
       </x:c>
       <x:c r="C61" s="5" t="str"/>
       <x:c r="D61" s="5" t="str"/>
@@ -3889,12 +4003,12 @@
       </x:c>
       <x:c r="H61" s="5" t="str"/>
       <x:c r="I61" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gilwern.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dinas.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="5" t="str">
-        <x:v>Gwernllwyn</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="B62" s="5" t="str">
         <x:v>Dowlais</x:v>
@@ -3910,36 +4024,38 @@
       </x:c>
       <x:c r="H62" s="5" t="str"/>
       <x:c r="I62" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gwernllwyn.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="5" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Dowlais (1851-1872)</x:v>
       </x:c>
       <x:c r="B63" s="5" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="C63" s="5" t="str"/>
       <x:c r="D63" s="5" t="str"/>
       <x:c r="E63" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F63" s="5" t="str"/>
+      <x:c r="F63" s="5" t="str">
+        <x:v>1851-1872</x:v>
+      </x:c>
       <x:c r="G63" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H63" s="5" t="str"/>
       <x:c r="I63" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Haverfordwest.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais_(1851-1872).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="5" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Ebbro Vale</x:v>
       </x:c>
       <x:c r="B64" s="5" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Ebbw Vale</x:v>
       </x:c>
       <x:c r="C64" s="5" t="str"/>
       <x:c r="D64" s="5" t="str"/>
@@ -3952,38 +4068,36 @@
       </x:c>
       <x:c r="H64" s="5" t="str"/>
       <x:c r="I64" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llandebie.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ebbro_Vale.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="5" t="str">
-        <x:v>Llanelli (1851-1867)</x:v>
+        <x:v>Ffestiniog</x:v>
       </x:c>
       <x:c r="B65" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Ffestiniog</x:v>
       </x:c>
       <x:c r="C65" s="5" t="str"/>
       <x:c r="D65" s="5" t="str"/>
       <x:c r="E65" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F65" s="5" t="str">
-        <x:v>1851-1867</x:v>
-      </x:c>
+      <x:c r="F65" s="5" t="str"/>
       <x:c r="G65" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H65" s="5" t="str"/>
       <x:c r="I65" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelli_(1851-1867).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ffestiniog.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Georgetown</x:v>
       </x:c>
       <x:c r="B66" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Georgetown</x:v>
       </x:c>
       <x:c r="C66" s="5" t="str"/>
       <x:c r="D66" s="5" t="str"/>
@@ -3996,84 +4110,78 @@
       </x:c>
       <x:c r="H66" s="5" t="str"/>
       <x:c r="I66" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelltyd.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Georgetown.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="5" t="str">
-        <x:v>Llanelly (1847-1849)</x:v>
+        <x:v>Gilwern</x:v>
       </x:c>
       <x:c r="B67" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Gilwern</x:v>
       </x:c>
       <x:c r="C67" s="5" t="str"/>
       <x:c r="D67" s="5" t="str"/>
       <x:c r="E67" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F67" s="5" t="str">
-        <x:v>1847-1849</x:v>
-      </x:c>
+      <x:c r="F67" s="5" t="str"/>
       <x:c r="G67" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H67" s="5" t="str"/>
       <x:c r="I67" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1849).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gilwern.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="5" t="str">
-        <x:v>Llanelly (1847-1868)</x:v>
+        <x:v>Gwernllwyn</x:v>
       </x:c>
       <x:c r="B68" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="C68" s="5" t="str"/>
       <x:c r="D68" s="5" t="str"/>
       <x:c r="E68" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F68" s="5" t="str">
-        <x:v>1847-1868</x:v>
-      </x:c>
+      <x:c r="F68" s="5" t="str"/>
       <x:c r="G68" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H68" s="5" t="str"/>
       <x:c r="I68" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1868).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gwernllwyn.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="5" t="str">
-        <x:v>Llanelly (1857-1863)</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="B69" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="C69" s="5" t="str"/>
       <x:c r="D69" s="5" t="str"/>
       <x:c r="E69" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F69" s="5" t="str">
-        <x:v>1857-1863</x:v>
-      </x:c>
+      <x:c r="F69" s="5" t="str"/>
       <x:c r="G69" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H69" s="5" t="str"/>
       <x:c r="I69" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1857-1863).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Haverfordwest.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="5" t="str">
-        <x:v>Llanelly 2</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="B70" s="5" t="str">
-        <x:v>Llanelly 2</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="C70" s="5" t="str"/>
       <x:c r="D70" s="5" t="str"/>
@@ -4086,36 +4194,38 @@
       </x:c>
       <x:c r="H70" s="5" t="str"/>
       <x:c r="I70" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_2.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llandebie.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="5" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Llanelli (1851-1867)</x:v>
       </x:c>
       <x:c r="B71" s="5" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C71" s="5" t="str"/>
       <x:c r="D71" s="5" t="str"/>
       <x:c r="E71" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F71" s="5" t="str"/>
+      <x:c r="F71" s="5" t="str">
+        <x:v>1851-1867</x:v>
+      </x:c>
       <x:c r="G71" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H71" s="5" t="str"/>
       <x:c r="I71" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanfabon.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelli_(1851-1867).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="B72" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="C72" s="5" t="str"/>
       <x:c r="D72" s="5" t="str"/>
@@ -4128,15 +4238,15 @@
       </x:c>
       <x:c r="H72" s="5" t="str"/>
       <x:c r="I72" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llansawel.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelltyd.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="5" t="str">
-        <x:v>Machen (1854-1865)</x:v>
+        <x:v>Llanelly (1847-1849)</x:v>
       </x:c>
       <x:c r="B73" s="5" t="str">
-        <x:v>Machen</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C73" s="5" t="str"/>
       <x:c r="D73" s="5" t="str"/>
@@ -4144,22 +4254,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F73" s="5" t="str">
-        <x:v>1854-1865</x:v>
+        <x:v>1847-1849</x:v>
       </x:c>
       <x:c r="G73" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H73" s="5" t="str"/>
       <x:c r="I73" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Machen_(1854-1865).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1849).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="5" t="str">
-        <x:v>Merthyr Tydfil (1843-1856)</x:v>
+        <x:v>Llanelly (1847-1868)</x:v>
       </x:c>
       <x:c r="B74" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C74" s="5" t="str"/>
       <x:c r="D74" s="5" t="str"/>
@@ -4167,22 +4277,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F74" s="5" t="str">
-        <x:v>1843-1856</x:v>
+        <x:v>1847-1868</x:v>
       </x:c>
       <x:c r="G74" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H74" s="5" t="str"/>
       <x:c r="I74" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1843-1856).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1868).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="5" t="str">
-        <x:v>Merthyr Tydfil (1861-1896)</x:v>
+        <x:v>Llanelly (1857-1863)</x:v>
       </x:c>
       <x:c r="B75" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C75" s="5" t="str"/>
       <x:c r="D75" s="5" t="str"/>
@@ -4190,68 +4300,64 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F75" s="5" t="str">
-        <x:v>1861-1896</x:v>
+        <x:v>1857-1863</x:v>
       </x:c>
       <x:c r="G75" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H75" s="5" t="str"/>
       <x:c r="I75" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1861-1896).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1857-1863).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="5" t="str">
-        <x:v>Merthyr Tydfil (1932-1943)</x:v>
+        <x:v>Llanelly 2</x:v>
       </x:c>
       <x:c r="B76" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Llanelly 2</x:v>
       </x:c>
       <x:c r="C76" s="5" t="str"/>
       <x:c r="D76" s="5" t="str"/>
       <x:c r="E76" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F76" s="5" t="str">
-        <x:v>1932-1943</x:v>
-      </x:c>
+      <x:c r="F76" s="5" t="str"/>
       <x:c r="G76" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H76" s="5" t="str"/>
       <x:c r="I76" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1932-1943).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_2.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="5" t="str">
-        <x:v>Merthyr Tydfil (Early to 1847)</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="B77" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="C77" s="5" t="str"/>
       <x:c r="D77" s="5" t="str"/>
       <x:c r="E77" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F77" s="5" t="str">
-        <x:v>1847</x:v>
-      </x:c>
+      <x:c r="F77" s="5" t="str"/>
       <x:c r="G77" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H77" s="5" t="str"/>
       <x:c r="I77" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(Early_to_1847).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanfabon.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="5" t="str">
-        <x:v>Nanty Glo</x:v>
+        <x:v>Llansawel</x:v>
       </x:c>
       <x:c r="B78" s="5" t="str">
-        <x:v>Nantyglo</x:v>
+        <x:v>Llansawel</x:v>
       </x:c>
       <x:c r="C78" s="5" t="str"/>
       <x:c r="D78" s="5" t="str"/>
@@ -4264,36 +4370,38 @@
       </x:c>
       <x:c r="H78" s="5" t="str"/>
       <x:c r="I78" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Nanty_Glo.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llansawel.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="5" t="str">
-        <x:v>Neath</x:v>
+        <x:v>Machen (1854-1865)</x:v>
       </x:c>
       <x:c r="B79" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Machen</x:v>
       </x:c>
       <x:c r="C79" s="5" t="str"/>
       <x:c r="D79" s="5" t="str"/>
       <x:c r="E79" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F79" s="5" t="str"/>
+      <x:c r="F79" s="5" t="str">
+        <x:v>1854-1865</x:v>
+      </x:c>
       <x:c r="G79" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H79" s="5" t="str"/>
       <x:c r="I79" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Neath.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Machen_(1854-1865).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="5" t="str">
-        <x:v>Pen-Y-Cae (1844-1866)</x:v>
+        <x:v>Merthyr Tydfil (1843-1856)</x:v>
       </x:c>
       <x:c r="B80" s="5" t="str">
-        <x:v>Pen-y-cae</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C80" s="5" t="str"/>
       <x:c r="D80" s="5" t="str"/>
@@ -4301,22 +4409,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F80" s="5" t="str">
-        <x:v>1844-1866</x:v>
+        <x:v>1843-1856</x:v>
       </x:c>
       <x:c r="G80" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H80" s="5" t="str"/>
       <x:c r="I80" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pen-Y-Cae_(1844-1866).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1843-1856).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="5" t="str">
-        <x:v>Pontlanfraith (Early to 1947)</x:v>
+        <x:v>Merthyr Tydfil (1861-1896)</x:v>
       </x:c>
       <x:c r="B81" s="5" t="str">
-        <x:v>Pontlanfraith</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C81" s="5" t="str"/>
       <x:c r="D81" s="5" t="str"/>
@@ -4324,22 +4432,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F81" s="5" t="str">
-        <x:v>1947</x:v>
+        <x:v>1861-1896</x:v>
       </x:c>
       <x:c r="G81" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H81" s="5" t="str"/>
       <x:c r="I81" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontlanfraith_(Early_to_1947).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1861-1896).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="5" t="str">
-        <x:v>Pontypridd (1877-1895)</x:v>
+        <x:v>Merthyr Tydfil (1932-1943)</x:v>
       </x:c>
       <x:c r="B82" s="5" t="str">
-        <x:v>Pontypridd</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C82" s="5" t="str"/>
       <x:c r="D82" s="5" t="str"/>
@@ -4347,22 +4455,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F82" s="5" t="str">
-        <x:v>1877-1895</x:v>
+        <x:v>1932-1943</x:v>
       </x:c>
       <x:c r="G82" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H82" s="5" t="str"/>
       <x:c r="I82" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontypridd_(1877-1895).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1932-1943).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="5" t="str">
-        <x:v>Welsh Conference (1850-1922)</x:v>
+        <x:v>Merthyr Tydfil (Early to 1847)</x:v>
       </x:c>
       <x:c r="B83" s="5" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C83" s="5" t="str"/>
       <x:c r="D83" s="5" t="str"/>
@@ -4370,160 +4478,156 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F83" s="5" t="str">
-        <x:v>1850-1922</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="G83" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H83" s="5" t="str"/>
       <x:c r="I83" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Welsh_Conference_(1850-1922).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(Early_to_1847).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Nanty Glo</x:v>
       </x:c>
       <x:c r="B84" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Nantyglo</x:v>
       </x:c>
       <x:c r="C84" s="5" t="str"/>
       <x:c r="D84" s="5" t="str"/>
       <x:c r="E84" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F84" s="5" t="str">
-        <x:v>ca. 1846-1947</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F84" s="5" t="str"/>
       <x:c r="G84" s="5" t="str">
-        <x:v>Film 104168 Items 1-6</x:v>
-      </x:c>
-      <x:c r="H84" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I84" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H84" s="5" t="str"/>
+      <x:c r="I84" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Nanty_Glo.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="5" t="str">
-        <x:v>Cefncoedycymer</x:v>
+        <x:v>Neath</x:v>
       </x:c>
       <x:c r="B85" s="5" t="str">
-        <x:v>Cefn Coed-y-Cymmer</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="C85" s="5" t="str"/>
       <x:c r="D85" s="5" t="str"/>
       <x:c r="E85" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F85" s="5" t="str">
-        <x:v>1847-1864</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F85" s="5" t="str"/>
       <x:c r="G85" s="5" t="str">
-        <x:v>Film 104168 Item 7</x:v>
-      </x:c>
-      <x:c r="H85" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I85" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H85" s="5" t="str"/>
+      <x:c r="I85" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Neath.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="5" t="str">
-        <x:v>Coalbrook Vale</x:v>
+        <x:v>Pen-Y-Cae (1844-1866)</x:v>
       </x:c>
       <x:c r="B86" s="5" t="str">
-        <x:v>Coalbrookvale</x:v>
+        <x:v>Pen-y-cae</x:v>
       </x:c>
       <x:c r="C86" s="5" t="str"/>
       <x:c r="D86" s="5" t="str"/>
       <x:c r="E86" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F86" s="5" t="str">
-        <x:v>ca. 1856-1867</x:v>
+        <x:v>1844-1866</x:v>
       </x:c>
       <x:c r="G86" s="5" t="str">
-        <x:v>Film 104168 Item 8</x:v>
-      </x:c>
-      <x:c r="H86" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I86" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H86" s="5" t="str"/>
+      <x:c r="I86" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pen-Y-Cae_(1844-1866).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Pontlanfraith (Early to 1947)</x:v>
       </x:c>
       <x:c r="B87" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Pontlanfraith</x:v>
       </x:c>
       <x:c r="C87" s="5" t="str"/>
       <x:c r="D87" s="5" t="str"/>
       <x:c r="E87" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F87" s="5" t="str">
-        <x:v>ca. 1848-1876</x:v>
+        <x:v>1947</x:v>
       </x:c>
       <x:c r="G87" s="5" t="str">
-        <x:v>Film 104168 Item 9</x:v>
-      </x:c>
-      <x:c r="H87" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I87" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H87" s="5" t="str"/>
+      <x:c r="I87" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontlanfraith_(Early_to_1947).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="5" t="str">
-        <x:v>Crumlin</x:v>
+        <x:v>Pontypridd (1877-1895)</x:v>
       </x:c>
       <x:c r="B88" s="5" t="str">
-        <x:v>Crumlin</x:v>
+        <x:v>Pontypridd</x:v>
       </x:c>
       <x:c r="C88" s="5" t="str"/>
       <x:c r="D88" s="5" t="str"/>
       <x:c r="E88" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F88" s="5" t="str">
-        <x:v>ca. 1857-1862</x:v>
+        <x:v>1877-1895</x:v>
       </x:c>
       <x:c r="G88" s="5" t="str">
-        <x:v>Film 104168 Item 10</x:v>
-      </x:c>
-      <x:c r="H88" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I88" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H88" s="5" t="str"/>
+      <x:c r="I88" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontypridd_(1877-1895).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Welsh Conference (1850-1922)</x:v>
       </x:c>
       <x:c r="B89" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Welsh Conference</x:v>
       </x:c>
       <x:c r="C89" s="5" t="str"/>
       <x:c r="D89" s="5" t="str"/>
       <x:c r="E89" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F89" s="5" t="str">
-        <x:v>1849-1876</x:v>
+        <x:v>1850-1922</x:v>
       </x:c>
       <x:c r="G89" s="5" t="str">
-        <x:v>Film 104168 Item 11</x:v>
-      </x:c>
-      <x:c r="H89" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I89" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H89" s="5" t="str"/>
+      <x:c r="I89" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Welsh_Conference_(1850-1922).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="5" t="str">
-        <x:v>Cwmcillyn</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="B90" s="5" t="str">
-        <x:v>Cwmcillyn</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C90" s="5" t="str"/>
       <x:c r="D90" s="5" t="str"/>
@@ -4531,10 +4635,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F90" s="5" t="str">
-        <x:v>1847-1856</x:v>
+        <x:v>ca. 1846-1947</x:v>
       </x:c>
       <x:c r="G90" s="5" t="str">
-        <x:v>Film 104168 Item 12</x:v>
+        <x:v>Film 104168 Items 1-6</x:v>
       </x:c>
       <x:c r="H90" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
@@ -4543,10 +4647,10 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="5" t="str">
-        <x:v>Cwmbran</x:v>
+        <x:v>Cefncoedycymer</x:v>
       </x:c>
       <x:c r="B91" s="5" t="str">
-        <x:v>Cwmbran</x:v>
+        <x:v>Cefn Coed-y-Cymmer</x:v>
       </x:c>
       <x:c r="C91" s="5" t="str"/>
       <x:c r="D91" s="5" t="str"/>
@@ -4554,10 +4658,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F91" s="5" t="str">
-        <x:v>1850-1874</x:v>
+        <x:v>1847-1864</x:v>
       </x:c>
       <x:c r="G91" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
+        <x:v>Film 104168 Item 7</x:v>
       </x:c>
       <x:c r="H91" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
@@ -4566,10 +4670,10 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="5" t="str">
-        <x:v>Llanelltud</x:v>
+        <x:v>Coalbrook Vale</x:v>
       </x:c>
       <x:c r="B92" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Coalbrookvale</x:v>
       </x:c>
       <x:c r="C92" s="5" t="str"/>
       <x:c r="D92" s="5" t="str"/>
@@ -4577,10 +4681,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F92" s="5" t="str">
-        <x:v>1850-1874</x:v>
+        <x:v>ca. 1856-1867</x:v>
       </x:c>
       <x:c r="G92" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
+        <x:v>Film 104168 Item 8</x:v>
       </x:c>
       <x:c r="H92" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
@@ -4589,10 +4693,10 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="B93" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="C93" s="5" t="str"/>
       <x:c r="D93" s="5" t="str"/>
@@ -4600,10 +4704,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F93" s="5" t="str">
-        <x:v>1875-1882</x:v>
+        <x:v>ca. 1848-1876</x:v>
       </x:c>
       <x:c r="G93" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
+        <x:v>Film 104168 Item 9</x:v>
       </x:c>
       <x:c r="H93" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
@@ -4612,10 +4716,10 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="5" t="str">
-        <x:v>Treboeth</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="B94" s="5" t="str">
-        <x:v>Treboeth</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="C94" s="5" t="str"/>
       <x:c r="D94" s="5" t="str"/>
@@ -4623,22 +4727,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F94" s="5" t="str">
-        <x:v>1844-1880</x:v>
+        <x:v>ca. 1857-1862</x:v>
       </x:c>
       <x:c r="G94" s="5" t="str">
-        <x:v>Film 104172 Item 1</x:v>
+        <x:v>Film 104168 Item 10</x:v>
       </x:c>
       <x:c r="H94" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I94" s="5" t="str"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="5" t="str">
-        <x:v>Tredegar</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="B95" s="5" t="str">
-        <x:v>Tredegar</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="C95" s="5" t="str"/>
       <x:c r="D95" s="5" t="str"/>
@@ -4646,22 +4750,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F95" s="5" t="str">
-        <x:v>ca. 1844-1883</x:v>
+        <x:v>1849-1876</x:v>
       </x:c>
       <x:c r="G95" s="5" t="str">
-        <x:v>Film 104172 Items 2-3</x:v>
+        <x:v>Film 104168 Item 11</x:v>
       </x:c>
       <x:c r="H95" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I95" s="5" t="str"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="5" t="str">
-        <x:v>Treforest</x:v>
+        <x:v>Cwmcillyn</x:v>
       </x:c>
       <x:c r="B96" s="5" t="str">
-        <x:v>Treforest</x:v>
+        <x:v>Cwmcillyn</x:v>
       </x:c>
       <x:c r="C96" s="5" t="str"/>
       <x:c r="D96" s="5" t="str"/>
@@ -4669,22 +4773,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F96" s="5" t="str">
-        <x:v>1851-1873</x:v>
+        <x:v>1847-1856</x:v>
       </x:c>
       <x:c r="G96" s="5" t="str">
-        <x:v>Film 104172 Item 4</x:v>
+        <x:v>Film 104168 Item 12</x:v>
       </x:c>
       <x:c r="H96" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I96" s="5" t="str"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="5" t="str">
-        <x:v>Morriston</x:v>
+        <x:v>Cwmbran</x:v>
       </x:c>
       <x:c r="B97" s="5" t="str">
-        <x:v>Morriston</x:v>
+        <x:v>Cwmbran</x:v>
       </x:c>
       <x:c r="C97" s="5" t="str"/>
       <x:c r="D97" s="5" t="str"/>
@@ -4692,22 +4796,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F97" s="5" t="str">
-        <x:v>1853-1868</x:v>
+        <x:v>1850-1874</x:v>
       </x:c>
       <x:c r="G97" s="5" t="str">
-        <x:v>Film 104172 Item 5</x:v>
+        <x:v>Film 104168 Item 13</x:v>
       </x:c>
       <x:c r="H97" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I97" s="5" t="str"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Llanelltud</x:v>
       </x:c>
       <x:c r="B98" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="C98" s="5" t="str"/>
       <x:c r="D98" s="5" t="str"/>
@@ -4715,22 +4819,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F98" s="5" t="str">
-        <x:v>1875-1882</x:v>
+        <x:v>1850-1874</x:v>
       </x:c>
       <x:c r="G98" s="5" t="str">
-        <x:v>Film 104172 Item 6</x:v>
+        <x:v>Film 104168 Item 13</x:v>
       </x:c>
       <x:c r="H98" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I98" s="5" t="str"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="5" t="str">
-        <x:v>Trinant</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="B99" s="5" t="str">
-        <x:v>Trinant</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="C99" s="5" t="str"/>
       <x:c r="D99" s="5" t="str"/>
@@ -4738,22 +4842,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F99" s="5" t="str">
-        <x:v>ca. 1849-1853</x:v>
+        <x:v>1875-1882</x:v>
       </x:c>
       <x:c r="G99" s="5" t="str">
-        <x:v>Film 104172 Item 6</x:v>
+        <x:v>Film 104168 Item 13</x:v>
       </x:c>
       <x:c r="H99" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I99" s="5" t="str"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="5" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Treboeth</x:v>
       </x:c>
       <x:c r="B100" s="5" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Treboeth</x:v>
       </x:c>
       <x:c r="C100" s="5" t="str"/>
       <x:c r="D100" s="5" t="str"/>
@@ -4761,10 +4865,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F100" s="5" t="str">
-        <x:v>1851-1883</x:v>
+        <x:v>1844-1880</x:v>
       </x:c>
       <x:c r="G100" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
+        <x:v>Film 104172 Item 1</x:v>
       </x:c>
       <x:c r="H100" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
@@ -4773,10 +4877,10 @@
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="5" t="str">
-        <x:v>Twyncarno</x:v>
+        <x:v>Tredegar</x:v>
       </x:c>
       <x:c r="B101" s="5" t="str">
-        <x:v>Twyncarno</x:v>
+        <x:v>Tredegar</x:v>
       </x:c>
       <x:c r="C101" s="5" t="str"/>
       <x:c r="D101" s="5" t="str"/>
@@ -4784,10 +4888,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F101" s="5" t="str">
-        <x:v>1851-1883</x:v>
+        <x:v>ca. 1844-1883</x:v>
       </x:c>
       <x:c r="G101" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
+        <x:v>Film 104172 Items 2-3</x:v>
       </x:c>
       <x:c r="H101" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
@@ -4796,10 +4900,10 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="5" t="str">
-        <x:v>Twyn-yr-Odyn</x:v>
+        <x:v>Treforest</x:v>
       </x:c>
       <x:c r="B102" s="5" t="str">
-        <x:v>Twyn-yr-Odyn</x:v>
+        <x:v>Treforest</x:v>
       </x:c>
       <x:c r="C102" s="5" t="str"/>
       <x:c r="D102" s="5" t="str"/>
@@ -4807,10 +4911,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F102" s="5" t="str">
-        <x:v>1847-1901</x:v>
+        <x:v>1851-1873</x:v>
       </x:c>
       <x:c r="G102" s="5" t="str">
-        <x:v>Film 104172 Items 9-10</x:v>
+        <x:v>Film 104172 Item 4</x:v>
       </x:c>
       <x:c r="H102" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
@@ -4819,10 +4923,10 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="5" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Morriston</x:v>
       </x:c>
       <x:c r="B103" s="5" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Morriston</x:v>
       </x:c>
       <x:c r="C103" s="5" t="str"/>
       <x:c r="D103" s="5" t="str"/>
@@ -4830,10 +4934,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F103" s="5" t="str">
-        <x:v>ca. 1850-1922</x:v>
+        <x:v>1853-1868</x:v>
       </x:c>
       <x:c r="G103" s="5" t="str">
-        <x:v>Film 104172 Item 11</x:v>
+        <x:v>Film 104172 Item 5</x:v>
       </x:c>
       <x:c r="H103" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
@@ -4842,10 +4946,10 @@
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="5" t="str">
-        <x:v>Ystrad</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="B104" s="5" t="str">
-        <x:v>Ystrad</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="C104" s="5" t="str"/>
       <x:c r="D104" s="5" t="str"/>
@@ -4853,10 +4957,10 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F104" s="5" t="str">
-        <x:v>ca. 1885-1911</x:v>
+        <x:v>1875-1882</x:v>
       </x:c>
       <x:c r="G104" s="5" t="str">
-        <x:v>Film 104172 Item 12</x:v>
+        <x:v>Film 104172 Item 6</x:v>
       </x:c>
       <x:c r="H104" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
@@ -4865,10 +4969,10 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Trinant</x:v>
       </x:c>
       <x:c r="B105" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Trinant</x:v>
       </x:c>
       <x:c r="C105" s="5" t="str"/>
       <x:c r="D105" s="5" t="str"/>
@@ -4876,22 +4980,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F105" s="5" t="str">
-        <x:v>1849-1855; 1850-1853; 1879</x:v>
+        <x:v>ca. 1849-1853</x:v>
       </x:c>
       <x:c r="G105" s="5" t="str">
-        <x:v>Film 104169 items 14-15</x:v>
+        <x:v>Film 104172 Item 6</x:v>
       </x:c>
       <x:c r="H105" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
       <x:c r="I105" s="5" t="str"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="5" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Rhymney English</x:v>
       </x:c>
       <x:c r="B106" s="5" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Rhymney English</x:v>
       </x:c>
       <x:c r="C106" s="5" t="str"/>
       <x:c r="D106" s="5" t="str"/>
@@ -4899,20 +5003,158 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F106" s="5" t="str">
+        <x:v>1851-1883</x:v>
+      </x:c>
+      <x:c r="G106" s="5" t="str">
+        <x:v>Film 104172 Items 7-8</x:v>
+      </x:c>
+      <x:c r="H106" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I106" s="5" t="str"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="5" t="str">
+        <x:v>Twyncarno</x:v>
+      </x:c>
+      <x:c r="B107" s="5" t="str">
+        <x:v>Twyncarno</x:v>
+      </x:c>
+      <x:c r="C107" s="5" t="str"/>
+      <x:c r="D107" s="5" t="str"/>
+      <x:c r="E107" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F107" s="5" t="str">
+        <x:v>1851-1883</x:v>
+      </x:c>
+      <x:c r="G107" s="5" t="str">
+        <x:v>Film 104172 Items 7-8</x:v>
+      </x:c>
+      <x:c r="H107" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I107" s="5" t="str"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="5" t="str">
+        <x:v>Twyn-yr-Odyn</x:v>
+      </x:c>
+      <x:c r="B108" s="5" t="str">
+        <x:v>Twyn-yr-Odyn</x:v>
+      </x:c>
+      <x:c r="C108" s="5" t="str"/>
+      <x:c r="D108" s="5" t="str"/>
+      <x:c r="E108" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F108" s="5" t="str">
+        <x:v>1847-1901</x:v>
+      </x:c>
+      <x:c r="G108" s="5" t="str">
+        <x:v>Film 104172 Items 9-10</x:v>
+      </x:c>
+      <x:c r="H108" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I108" s="5" t="str"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="5" t="str">
+        <x:v>Welsh Conference</x:v>
+      </x:c>
+      <x:c r="B109" s="5" t="str">
+        <x:v>Welsh Conference</x:v>
+      </x:c>
+      <x:c r="C109" s="5" t="str"/>
+      <x:c r="D109" s="5" t="str"/>
+      <x:c r="E109" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F109" s="5" t="str">
+        <x:v>ca. 1850-1922</x:v>
+      </x:c>
+      <x:c r="G109" s="5" t="str">
+        <x:v>Film 104172 Item 11</x:v>
+      </x:c>
+      <x:c r="H109" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I109" s="5" t="str"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="5" t="str">
+        <x:v>Ystrad</x:v>
+      </x:c>
+      <x:c r="B110" s="5" t="str">
+        <x:v>Ystrad</x:v>
+      </x:c>
+      <x:c r="C110" s="5" t="str"/>
+      <x:c r="D110" s="5" t="str"/>
+      <x:c r="E110" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F110" s="5" t="str">
+        <x:v>ca. 1885-1911</x:v>
+      </x:c>
+      <x:c r="G110" s="5" t="str">
+        <x:v>Film 104172 Item 12</x:v>
+      </x:c>
+      <x:c r="H110" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I110" s="5" t="str"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="5" t="str">
+        <x:v>Llansawel</x:v>
+      </x:c>
+      <x:c r="B111" s="5" t="str">
+        <x:v>Llansawel</x:v>
+      </x:c>
+      <x:c r="C111" s="5" t="str"/>
+      <x:c r="D111" s="5" t="str"/>
+      <x:c r="E111" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F111" s="5" t="str">
+        <x:v>1849-1855; 1850-1853; 1879</x:v>
+      </x:c>
+      <x:c r="G111" s="5" t="str">
+        <x:v>Film 104169 items 14-15</x:v>
+      </x:c>
+      <x:c r="H111" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+      </x:c>
+      <x:c r="I111" s="5" t="str"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="5" t="str">
+        <x:v>Sutton Mountain</x:v>
+      </x:c>
+      <x:c r="B112" s="5" t="str">
+        <x:v>Sutton Mountain</x:v>
+      </x:c>
+      <x:c r="C112" s="5" t="str"/>
+      <x:c r="D112" s="5" t="str"/>
+      <x:c r="E112" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F112" s="5" t="str">
         <x:v>1853-1859</x:v>
       </x:c>
-      <x:c r="G106" s="5" t="str">
+      <x:c r="G112" s="5" t="str">
         <x:v>Film 104171 item 6</x:v>
       </x:c>
-      <x:c r="H106" s="5" t="str">
+      <x:c r="H112" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104171</x:v>
       </x:c>
-      <x:c r="I106" s="5" t="str"/>
+      <x:c r="I112" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e1bc452275140f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2ec2a70f4214540"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>